<commit_message>
Actualización automática 2026-09-24 11:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R101"/>
+  <dimension ref="A1:R102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3954,7 +3954,7 @@
         <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0</v>
+        <v>397.85</v>
       </c>
       <c r="M58" s="2" t="n">
         <v>0</v>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5022,10 +5022,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>358.2</v>
+        <v>0</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>551.99</v>
+        <v>0</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0</v>
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5082,10 +5082,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>0</v>
+        <v>358.2</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>0</v>
+        <v>551.99</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0</v>
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5397,7 +5397,7 @@
         <v>0</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>40.12</v>
+        <v>0</v>
       </c>
       <c r="N82" s="2" t="n">
         <v>0</v>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>TOCAGON PILA ANA ROSA</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5457,7 +5457,7 @@
         <v>0</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>0</v>
+        <v>40.12</v>
       </c>
       <c r="N83" s="2" t="n">
         <v>0</v>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TOCAGON PILA ANA ROSA</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5691,7 +5691,7 @@
         <v>0</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>90.23999999999999</v>
+        <v>0</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5751,7 +5751,7 @@
         <v>0</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>0</v>
+        <v>90.23999999999999</v>
       </c>
       <c r="L88" s="2" t="n">
         <v>0</v>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,137 +6443,197 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
+          <t>ZAZACORP S.A.</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R100" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
           <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
-      <c r="C100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R100" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="C101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="D101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="E101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="F101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="G101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="H101" s="3" t="inlineStr">
-        <is>
-          <t>3 de 99</t>
-        </is>
-      </c>
-      <c r="I101" s="3" t="inlineStr">
-        <is>
-          <t>3 de 99</t>
-        </is>
-      </c>
-      <c r="J101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="K101" s="3" t="inlineStr">
-        <is>
-          <t>3 de 99</t>
-        </is>
-      </c>
-      <c r="L101" s="3" t="inlineStr">
-        <is>
-          <t>1 de 99</t>
-        </is>
-      </c>
-      <c r="M101" s="3" t="inlineStr">
-        <is>
-          <t>4 de 99</t>
-        </is>
-      </c>
-      <c r="N101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="O101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="P101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="Q101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="R101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
+      <c r="C101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R101" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>0 de 100</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>0 de 100</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>0 de 100</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t>0 de 100</t>
+        </is>
+      </c>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>0 de 100</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>3 de 100</t>
+        </is>
+      </c>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
+          <t>3 de 100</t>
+        </is>
+      </c>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>0 de 100</t>
+        </is>
+      </c>
+      <c r="K102" s="3" t="inlineStr">
+        <is>
+          <t>3 de 100</t>
+        </is>
+      </c>
+      <c r="L102" s="3" t="inlineStr">
+        <is>
+          <t>2 de 100</t>
+        </is>
+      </c>
+      <c r="M102" s="3" t="inlineStr">
+        <is>
+          <t>4 de 100</t>
+        </is>
+      </c>
+      <c r="N102" s="3" t="inlineStr">
+        <is>
+          <t>0 de 100</t>
+        </is>
+      </c>
+      <c r="O102" s="3" t="inlineStr">
+        <is>
+          <t>0 de 100</t>
+        </is>
+      </c>
+      <c r="P102" s="3" t="inlineStr">
+        <is>
+          <t>0 de 100</t>
+        </is>
+      </c>
+      <c r="Q102" s="3" t="inlineStr">
+        <is>
+          <t>0 de 100</t>
+        </is>
+      </c>
+      <c r="R102" s="3" t="inlineStr">
+        <is>
+          <t>0 de 100</t>
         </is>
       </c>
     </row>
@@ -8818,7 +8878,7 @@
         <v>0</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>0</v>
+        <v>397.85</v>
       </c>
       <c r="G82" s="2" t="n">
         <v>0</v>
@@ -10401,7 +10461,7 @@
         <v>8971.120000000001</v>
       </c>
       <c r="F141" s="4" t="n">
-        <v>6505.610000000001</v>
+        <v>6903.46</v>
       </c>
       <c r="G141" s="4" t="n">
         <v>0</v>
@@ -10524,13 +10584,13 @@
         <v>7434</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>4150.73</v>
+        <v>4548.58</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3283.27</v>
+        <v>2885.42</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.5583440947000269</v>
+        <v>0.6118617164379876</v>
       </c>
     </row>
     <row r="5">
@@ -10567,13 +10627,13 @@
         <v>37067</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>21293.15</v>
+        <v>21691</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>15773.85</v>
+        <v>15376</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.5744503196913697</v>
+        <v>0.5851835864785389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-25 08:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R102"/>
+  <dimension ref="A1:R101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5022,10 +5022,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>0</v>
+        <v>358.2</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>0</v>
+        <v>551.99</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0</v>
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5082,10 +5082,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>358.2</v>
+        <v>0</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>551.99</v>
+        <v>0</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0</v>
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5397,7 +5397,7 @@
         <v>0</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>0</v>
+        <v>40.12</v>
       </c>
       <c r="N82" s="2" t="n">
         <v>0</v>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>TOCAGON PILA ANA ROSA</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5457,7 +5457,7 @@
         <v>0</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>40.12</v>
+        <v>0</v>
       </c>
       <c r="N83" s="2" t="n">
         <v>0</v>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TOCAGON PILA ANA ROSA</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5691,7 +5691,7 @@
         <v>0</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>0</v>
+        <v>90.23999999999999</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5751,7 +5751,7 @@
         <v>0</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>90.23999999999999</v>
+        <v>0</v>
       </c>
       <c r="L88" s="2" t="n">
         <v>0</v>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6496,144 +6496,84 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q101" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R101" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="C102" s="3" t="inlineStr">
-        <is>
-          <t>0 de 100</t>
-        </is>
-      </c>
-      <c r="D102" s="3" t="inlineStr">
-        <is>
-          <t>0 de 100</t>
-        </is>
-      </c>
-      <c r="E102" s="3" t="inlineStr">
-        <is>
-          <t>0 de 100</t>
-        </is>
-      </c>
-      <c r="F102" s="3" t="inlineStr">
-        <is>
-          <t>0 de 100</t>
-        </is>
-      </c>
-      <c r="G102" s="3" t="inlineStr">
-        <is>
-          <t>0 de 100</t>
-        </is>
-      </c>
-      <c r="H102" s="3" t="inlineStr">
-        <is>
-          <t>3 de 100</t>
-        </is>
-      </c>
-      <c r="I102" s="3" t="inlineStr">
-        <is>
-          <t>3 de 100</t>
-        </is>
-      </c>
-      <c r="J102" s="3" t="inlineStr">
-        <is>
-          <t>0 de 100</t>
-        </is>
-      </c>
-      <c r="K102" s="3" t="inlineStr">
-        <is>
-          <t>3 de 100</t>
-        </is>
-      </c>
-      <c r="L102" s="3" t="inlineStr">
-        <is>
-          <t>2 de 100</t>
-        </is>
-      </c>
-      <c r="M102" s="3" t="inlineStr">
-        <is>
-          <t>4 de 100</t>
-        </is>
-      </c>
-      <c r="N102" s="3" t="inlineStr">
-        <is>
-          <t>0 de 100</t>
-        </is>
-      </c>
-      <c r="O102" s="3" t="inlineStr">
-        <is>
-          <t>0 de 100</t>
-        </is>
-      </c>
-      <c r="P102" s="3" t="inlineStr">
-        <is>
-          <t>0 de 100</t>
-        </is>
-      </c>
-      <c r="Q102" s="3" t="inlineStr">
-        <is>
-          <t>0 de 100</t>
-        </is>
-      </c>
-      <c r="R102" s="3" t="inlineStr">
-        <is>
-          <t>0 de 100</t>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>0 de 99</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>0 de 99</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>0 de 99</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>0 de 99</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>0 de 99</t>
+        </is>
+      </c>
+      <c r="H101" s="3" t="inlineStr">
+        <is>
+          <t>3 de 99</t>
+        </is>
+      </c>
+      <c r="I101" s="3" t="inlineStr">
+        <is>
+          <t>3 de 99</t>
+        </is>
+      </c>
+      <c r="J101" s="3" t="inlineStr">
+        <is>
+          <t>0 de 99</t>
+        </is>
+      </c>
+      <c r="K101" s="3" t="inlineStr">
+        <is>
+          <t>3 de 99</t>
+        </is>
+      </c>
+      <c r="L101" s="3" t="inlineStr">
+        <is>
+          <t>2 de 99</t>
+        </is>
+      </c>
+      <c r="M101" s="3" t="inlineStr">
+        <is>
+          <t>4 de 99</t>
+        </is>
+      </c>
+      <c r="N101" s="3" t="inlineStr">
+        <is>
+          <t>0 de 99</t>
+        </is>
+      </c>
+      <c r="O101" s="3" t="inlineStr">
+        <is>
+          <t>0 de 99</t>
+        </is>
+      </c>
+      <c r="P101" s="3" t="inlineStr">
+        <is>
+          <t>0 de 99</t>
+        </is>
+      </c>
+      <c r="Q101" s="3" t="inlineStr">
+        <is>
+          <t>0 de 99</t>
+        </is>
+      </c>
+      <c r="R101" s="3" t="inlineStr">
+        <is>
+          <t>0 de 99</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-10-05 08:30:14
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R101"/>
+  <dimension ref="A1:R100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SANCHEZ JARA LISSETTE MARIA</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SANCHEZ JARA LISSETTE MARIA</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>TOCAGON PILA ANA ROSA</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TOCAGON PILA ANA ROSA</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6436,144 +6436,84 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R100" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="C101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="D101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="E101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="F101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="G101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="H101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="I101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="J101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="K101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="L101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="M101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="N101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="O101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="P101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="Q101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
-        </is>
-      </c>
-      <c r="R101" s="3" t="inlineStr">
-        <is>
-          <t>0 de 99</t>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="J100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="L100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="M100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="N100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="O100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="P100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="Q100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
+        </is>
+      </c>
+      <c r="R100" s="3" t="inlineStr">
+        <is>
+          <t>0 de 98</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-10-08 08:30:15
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R98"/>
+  <dimension ref="A1:R97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6256,144 +6256,84 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R97" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="C98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="D98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="E98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="F98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="G98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="H98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="I98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="J98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="K98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="L98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="M98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="N98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="O98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="P98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="Q98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
-        </is>
-      </c>
-      <c r="R98" s="3" t="inlineStr">
-        <is>
-          <t>0 de 96</t>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="K97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="L97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="M97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="N97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="O97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="P97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="Q97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="R97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-10-09 08:30:14
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R97"/>
+  <dimension ref="A1:R96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GITI ECUADOR CIA. LTDA.</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>GITI ECUADOR CIA. LTDA.</t>
+          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SANCHEZ JARA LISSETTE MARIA</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SANCHEZ JARA LISSETTE MARIA</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>TOCAGON PILA ANA ROSA</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>TOCAGON PILA ANA ROSA</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6196,144 +6196,84 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R96" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="C97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="D97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="E97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="F97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="G97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="H97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="I97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="J97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="K97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="L97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="M97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="N97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="O97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="P97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="Q97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
-        </is>
-      </c>
-      <c r="R97" s="3" t="inlineStr">
-        <is>
-          <t>0 de 95</t>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="K96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="L96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="M96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="N96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="O96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="P96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="Q96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
+        </is>
+      </c>
+      <c r="R96" s="3" t="inlineStr">
+        <is>
+          <t>0 de 94</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-10-13 12:30:14
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R96"/>
+  <dimension ref="A1:R97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SERRANO VERA ANGGY PAULINA</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5013,7 +5013,7 @@
         <v>0</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="F76" s="2" t="n">
         <v>0</v>
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>TOCAGON PILA ANA ROSA</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TOCAGON PILA ANA ROSA</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,137 +6143,197 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
+          <t>ZAZACORP S.A.</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R95" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
           <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
-      <c r="C95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q95" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R95" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="C96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="E96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="F96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="G96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="H96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="I96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="J96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="K96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="L96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="M96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="N96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="O96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="P96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="Q96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
-        </is>
-      </c>
-      <c r="R96" s="3" t="inlineStr">
-        <is>
-          <t>0 de 94</t>
+      <c r="C96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R96" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>1 de 95</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="K97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="L97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="M97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="N97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="O97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="P97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="Q97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
+        </is>
+      </c>
+      <c r="R97" s="3" t="inlineStr">
+        <is>
+          <t>0 de 95</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G143"/>
+  <dimension ref="A1:G144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9450,7 +9510,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>SILVA BLUM CARLOS ALFREDO</t>
+          <t>SERRANO VERA ANGGY PAULINA</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
@@ -9463,7 +9523,7 @@
         <v>0</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="G117" s="2" t="n">
         <v>0</v>
@@ -9477,7 +9537,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SILVA BLUM CARLOS ALFREDO</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
@@ -9504,7 +9564,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
@@ -9531,7 +9591,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
@@ -9558,7 +9618,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
@@ -9585,7 +9645,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
@@ -9612,17 +9672,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
-        <v>23.49</v>
+        <v>0</v>
       </c>
       <c r="D123" s="2" t="n">
-        <v>150.37</v>
+        <v>0</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>40.12</v>
+        <v>0</v>
       </c>
       <c r="F123" s="2" t="n">
         <v>0</v>
@@ -9639,17 +9699,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>TOCAGON PILA ANA ROSA</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
-        <v>0</v>
+        <v>23.49</v>
       </c>
       <c r="D124" s="2" t="n">
-        <v>120.45</v>
+        <v>150.37</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>0</v>
+        <v>40.12</v>
       </c>
       <c r="F124" s="2" t="n">
         <v>0</v>
@@ -9666,14 +9726,14 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TOCAGON PILA ANA ROSA</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D125" s="2" t="n">
-        <v>0</v>
+        <v>120.45</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>0</v>
@@ -9693,7 +9753,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
@@ -9720,7 +9780,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
@@ -9747,11 +9807,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
-        <v>147.45</v>
+        <v>0</v>
       </c>
       <c r="D128" s="2" t="n">
         <v>0</v>
@@ -9774,11 +9834,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
-        <v>0</v>
+        <v>147.45</v>
       </c>
       <c r="D129" s="2" t="n">
         <v>0</v>
@@ -9801,7 +9861,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
@@ -9828,7 +9888,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
@@ -9855,7 +9915,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
@@ -9882,7 +9942,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
@@ -9909,7 +9969,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
@@ -9936,7 +9996,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
@@ -9963,14 +10023,14 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D136" s="2" t="n">
-        <v>181.96</v>
+        <v>0</v>
       </c>
       <c r="E136" s="2" t="n">
         <v>0</v>
@@ -9990,14 +10050,14 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D137" s="2" t="n">
-        <v>0</v>
+        <v>181.96</v>
       </c>
       <c r="E137" s="2" t="n">
         <v>0</v>
@@ -10017,7 +10077,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
@@ -10044,7 +10104,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
@@ -10071,7 +10131,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
@@ -10098,7 +10158,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
@@ -10108,7 +10168,7 @@
         <v>0</v>
       </c>
       <c r="E141" s="2" t="n">
-        <v>31.18</v>
+        <v>0</v>
       </c>
       <c r="F141" s="2" t="n">
         <v>0</v>
@@ -10125,39 +10185,66 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" s="2" t="n">
+        <v>31.18</v>
+      </c>
+      <c r="F142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
           <t>ZUÑIGA BUSTAMANTE ENRIQUE HAMLET</t>
         </is>
       </c>
-      <c r="C142" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D142" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E142" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F142" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G142" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="C143" s="4" t="n">
+      <c r="C143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="C144" s="4" t="n">
         <v>5045.25</v>
       </c>
-      <c r="D143" s="4" t="n">
+      <c r="D144" s="4" t="n">
         <v>9479.030000000001</v>
       </c>
-      <c r="E143" s="4" t="n">
+      <c r="E144" s="4" t="n">
         <v>11108.99</v>
       </c>
-      <c r="F143" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G143" s="4" t="n">
+      <c r="F144" s="4" t="n">
+        <v>107.46</v>
+      </c>
+      <c r="G144" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-10-27 09:30:17
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -4671,7 +4671,7 @@
         <v>0</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>214.32</v>
+        <v>321.48</v>
       </c>
       <c r="L70" s="2" t="n">
         <v>0</v>
@@ -9406,7 +9406,7 @@
         <v>0</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>214.32</v>
+        <v>321.48</v>
       </c>
       <c r="G106" s="2" t="n">
         <v>0</v>
@@ -10503,7 +10503,7 @@
         <v>11108.99</v>
       </c>
       <c r="F147" s="4" t="n">
-        <v>4116.68</v>
+        <v>4223.84</v>
       </c>
       <c r="G147" s="4" t="n">
         <v>0</v>
@@ -10602,10 +10602,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1903.93</v>
+        <v>2011.09</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-1903.93</v>
+        <v>-2011.09</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -10669,13 +10669,13 @@
         <v>46104</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>17548.21</v>
+        <v>17655.37</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>28555.79</v>
+        <v>28448.63</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.3806222887385042</v>
+        <v>0.3829465989935797</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-30 11:30:17
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -10602,10 +10602,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2880.77</v>
+        <v>2898.03</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-2880.77</v>
+        <v>-2898.03</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -10669,13 +10669,13 @@
         <v>46104</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>25523.58</v>
+        <v>25540.84</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>20580.42</v>
+        <v>20563.16</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.5536087975013013</v>
+        <v>0.5539831684886344</v>
       </c>
     </row>
   </sheetData>

</xml_diff>